<commit_message>
Se realizan varios ajustes
</commit_message>
<xml_diff>
--- a/database/seeders/Files/areas.xlsx
+++ b/database/seeders/Files/areas.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\sw_citca\database\seeders\Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\sw_CITCA\database\seeders\Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE6C5FAF-5073-4B13-AE80-07639065DB7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23985" windowHeight="8955"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="areas" sheetId="1" r:id="rId1"/>
@@ -20,31 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="69">
-  <si>
-    <t>Física, Matemáticas y Ciencias de la Tierra</t>
-  </si>
-  <si>
-    <t>Biología y Química</t>
-  </si>
-  <si>
-    <t>Medicina y Salud</t>
-  </si>
-  <si>
-    <t>Biotecnología y Ciencias Agropecuarias</t>
-  </si>
-  <si>
-    <t>Tecnología 4.0</t>
-  </si>
-  <si>
-    <t>Ingeniería e Industria</t>
-  </si>
-  <si>
-    <t>Ciencias Sociales</t>
-  </si>
-  <si>
-    <t>Interdisciplinaria (Litio, Ferroviarios, Semiconductores)</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="80">
   <si>
     <t>Astrofísica</t>
   </si>
@@ -227,12 +204,69 @@
   </si>
   <si>
     <t>parent_id</t>
+  </si>
+  <si>
+    <t>Ingeniería Electrónica</t>
+  </si>
+  <si>
+    <t>Ingeniería Mecánica</t>
+  </si>
+  <si>
+    <t>Ingeniería Mecatrónica</t>
+  </si>
+  <si>
+    <t>Ciencias Computacionales</t>
+  </si>
+  <si>
+    <t>Ciencias de la Ingeniería</t>
+  </si>
+  <si>
+    <t>Otras Ingenierías</t>
+  </si>
+  <si>
+    <t>Electromovilidad</t>
+  </si>
+  <si>
+    <t>Desarrollo Sostenible</t>
+  </si>
+  <si>
+    <t>Cambio Climático</t>
+  </si>
+  <si>
+    <t>Economía Circular</t>
+  </si>
+  <si>
+    <t>Gestión del Agua</t>
+  </si>
+  <si>
+    <t>Educación y Cultura</t>
+  </si>
+  <si>
+    <t>Tecnología 5.0 y Ciencia de Datos</t>
+  </si>
+  <si>
+    <t>Sistemas Socioecológicos</t>
+  </si>
+  <si>
+    <t>Vivienda</t>
+  </si>
+  <si>
+    <t>Sistemas agroalimentarios sustentables</t>
+  </si>
+  <si>
+    <t>Salud</t>
+  </si>
+  <si>
+    <t>Eficiencia Energética/Energías Renovables</t>
+  </si>
+  <si>
+    <t>Agentes Tóxicos y Procesos Contaminantes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -714,48 +748,48 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Buena" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Cálculo" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Celda de comprobación" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Celda vinculada" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Encabezado 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Encabezado 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Énfasis1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Énfasis2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Énfasis3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Énfasis4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Énfasis5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Énfasis6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Incorrecto" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Notas" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Salida" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Texto de advertencia" xfId="14" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="Texto explicativo" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Título" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Título 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Título 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1066,724 +1100,983 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C67"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C90"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="49.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="B1" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="C1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>9</v>
+        <v>72</v>
       </c>
       <c r="C11">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B12" t="s">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="C13">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B14" t="s">
-        <v>12</v>
+        <v>73</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>13</v>
+        <v>74</v>
       </c>
       <c r="C15">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B16" t="s">
-        <v>14</v>
+        <v>75</v>
       </c>
       <c r="C16">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>15</v>
+        <v>76</v>
       </c>
       <c r="C17">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B18" t="s">
-        <v>16</v>
+        <v>77</v>
       </c>
       <c r="C18">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B19" t="s">
+        <v>71</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>13</v>
+      </c>
+      <c r="B20" t="s">
+        <v>78</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21">
         <v>14</v>
       </c>
-      <c r="C19">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>11</v>
-      </c>
-      <c r="B20" t="s">
-        <v>17</v>
-      </c>
-      <c r="C20">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21">
-        <v>12</v>
-      </c>
       <c r="B21" t="s">
-        <v>18</v>
+        <v>79</v>
       </c>
       <c r="C21">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B22" t="s">
-        <v>19</v>
+        <v>69</v>
       </c>
       <c r="C22">
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B23" t="s">
-        <v>20</v>
+        <v>70</v>
       </c>
       <c r="C23">
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B24" t="s">
+        <v>68</v>
+      </c>
+      <c r="C24">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>18</v>
+      </c>
+      <c r="B25" t="s">
+        <v>72</v>
+      </c>
+      <c r="C25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>19</v>
+      </c>
+      <c r="B26" t="s">
+        <v>67</v>
+      </c>
+      <c r="C26">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>20</v>
+      </c>
+      <c r="B27" t="s">
+        <v>31</v>
+      </c>
+      <c r="C27">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28">
         <v>21</v>
       </c>
-      <c r="C24">
+      <c r="B28" t="s">
+        <v>73</v>
+      </c>
+      <c r="C28">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>22</v>
+      </c>
+      <c r="B29" t="s">
+        <v>74</v>
+      </c>
+      <c r="C29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>23</v>
+      </c>
+      <c r="B30" t="s">
+        <v>75</v>
+      </c>
+      <c r="C30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>24</v>
+      </c>
+      <c r="B31" t="s">
+        <v>76</v>
+      </c>
+      <c r="C31">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>25</v>
+      </c>
+      <c r="B32" t="s">
+        <v>77</v>
+      </c>
+      <c r="C32">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>26</v>
+      </c>
+      <c r="B33" t="s">
+        <v>71</v>
+      </c>
+      <c r="C33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>27</v>
+      </c>
+      <c r="B34" t="s">
+        <v>78</v>
+      </c>
+      <c r="C34">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>28</v>
+      </c>
+      <c r="B35" t="s">
+        <v>79</v>
+      </c>
+      <c r="C35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>29</v>
+      </c>
+      <c r="B36" t="s">
+        <v>69</v>
+      </c>
+      <c r="C36">
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25">
-        <v>16</v>
-      </c>
-      <c r="B25" t="s">
-        <v>22</v>
-      </c>
-      <c r="C25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>30</v>
+      </c>
+      <c r="B37" t="s">
+        <v>70</v>
+      </c>
+      <c r="C37">
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>17</v>
-      </c>
-      <c r="B26" t="s">
-        <v>23</v>
-      </c>
-      <c r="C26">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>31</v>
+      </c>
+      <c r="B38" t="s">
+        <v>68</v>
+      </c>
+      <c r="C38">
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27">
-        <v>18</v>
-      </c>
-      <c r="B27" t="s">
-        <v>24</v>
-      </c>
-      <c r="C27">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>32</v>
+      </c>
+      <c r="B39" t="s">
+        <v>72</v>
+      </c>
+      <c r="C39">
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28">
-        <v>19</v>
-      </c>
-      <c r="B28" t="s">
-        <v>25</v>
-      </c>
-      <c r="C28">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>33</v>
+      </c>
+      <c r="B40" t="s">
+        <v>67</v>
+      </c>
+      <c r="C40">
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29">
-        <v>20</v>
-      </c>
-      <c r="B29" t="s">
-        <v>26</v>
-      </c>
-      <c r="C29">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>34</v>
+      </c>
+      <c r="B41" t="s">
+        <v>31</v>
+      </c>
+      <c r="C41">
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30">
-        <v>21</v>
-      </c>
-      <c r="B30" t="s">
-        <v>27</v>
-      </c>
-      <c r="C30">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>35</v>
+      </c>
+      <c r="B42" t="s">
+        <v>73</v>
+      </c>
+      <c r="C42">
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31">
-        <v>22</v>
-      </c>
-      <c r="B31" t="s">
-        <v>28</v>
-      </c>
-      <c r="C31">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>36</v>
+      </c>
+      <c r="B43" t="s">
+        <v>74</v>
+      </c>
+      <c r="C43">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>37</v>
+      </c>
+      <c r="B44" t="s">
+        <v>75</v>
+      </c>
+      <c r="C44">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <v>38</v>
+      </c>
+      <c r="B45" t="s">
+        <v>76</v>
+      </c>
+      <c r="C45">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <v>39</v>
+      </c>
+      <c r="B46" t="s">
+        <v>77</v>
+      </c>
+      <c r="C46">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47">
+        <v>40</v>
+      </c>
+      <c r="B47" t="s">
+        <v>71</v>
+      </c>
+      <c r="C47">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <v>41</v>
+      </c>
+      <c r="B48" t="s">
+        <v>78</v>
+      </c>
+      <c r="C48">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <v>42</v>
+      </c>
+      <c r="B49" t="s">
+        <v>79</v>
+      </c>
+      <c r="C49">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>43</v>
+      </c>
+      <c r="B50" t="s">
+        <v>69</v>
+      </c>
+      <c r="C50">
         <v>4</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32">
-        <v>23</v>
-      </c>
-      <c r="B32" t="s">
-        <v>29</v>
-      </c>
-      <c r="C32">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>44</v>
+      </c>
+      <c r="B51" t="s">
+        <v>70</v>
+      </c>
+      <c r="C51">
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33">
-        <v>24</v>
-      </c>
-      <c r="B33" t="s">
-        <v>30</v>
-      </c>
-      <c r="C33">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <v>45</v>
+      </c>
+      <c r="B52" t="s">
+        <v>68</v>
+      </c>
+      <c r="C52">
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34">
-        <v>25</v>
-      </c>
-      <c r="B34" t="s">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53">
+        <v>46</v>
+      </c>
+      <c r="B53" t="s">
+        <v>72</v>
+      </c>
+      <c r="C53">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A54">
+        <v>47</v>
+      </c>
+      <c r="B54" t="s">
+        <v>67</v>
+      </c>
+      <c r="C54">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55">
+        <v>48</v>
+      </c>
+      <c r="B55" t="s">
         <v>31</v>
       </c>
-      <c r="C34">
+      <c r="C55">
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35">
-        <v>26</v>
-      </c>
-      <c r="B35" t="s">
-        <v>32</v>
-      </c>
-      <c r="C35">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A56">
+        <v>49</v>
+      </c>
+      <c r="B56" t="s">
+        <v>73</v>
+      </c>
+      <c r="C56">
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36">
-        <v>27</v>
-      </c>
-      <c r="B36" t="s">
-        <v>33</v>
-      </c>
-      <c r="C36">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A57">
+        <v>50</v>
+      </c>
+      <c r="B57" t="s">
+        <v>74</v>
+      </c>
+      <c r="C57">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A58">
+        <v>51</v>
+      </c>
+      <c r="B58" t="s">
+        <v>75</v>
+      </c>
+      <c r="C58">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A59">
+        <v>52</v>
+      </c>
+      <c r="B59" t="s">
+        <v>76</v>
+      </c>
+      <c r="C59">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A60">
+        <v>53</v>
+      </c>
+      <c r="B60" t="s">
+        <v>77</v>
+      </c>
+      <c r="C60">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A61">
+        <v>54</v>
+      </c>
+      <c r="B61" t="s">
+        <v>71</v>
+      </c>
+      <c r="C61">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A62">
+        <v>55</v>
+      </c>
+      <c r="B62" t="s">
+        <v>78</v>
+      </c>
+      <c r="C62">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A63">
+        <v>56</v>
+      </c>
+      <c r="B63" t="s">
+        <v>79</v>
+      </c>
+      <c r="C63">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A64">
+        <v>57</v>
+      </c>
+      <c r="B64" t="s">
+        <v>69</v>
+      </c>
+      <c r="C64">
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37">
-        <v>28</v>
-      </c>
-      <c r="B37" t="s">
-        <v>34</v>
-      </c>
-      <c r="C37">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65">
+        <v>58</v>
+      </c>
+      <c r="B65" t="s">
+        <v>70</v>
+      </c>
+      <c r="C65">
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38">
-        <v>29</v>
-      </c>
-      <c r="B38" t="s">
-        <v>35</v>
-      </c>
-      <c r="C38">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A66">
+        <v>59</v>
+      </c>
+      <c r="B66" t="s">
+        <v>68</v>
+      </c>
+      <c r="C66">
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39">
-        <v>30</v>
-      </c>
-      <c r="B39" t="s">
-        <v>36</v>
-      </c>
-      <c r="C39">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67">
+        <v>60</v>
+      </c>
+      <c r="B67" t="s">
+        <v>72</v>
+      </c>
+      <c r="C67">
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68">
+        <v>61</v>
+      </c>
+      <c r="B68" t="s">
+        <v>67</v>
+      </c>
+      <c r="C68">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A69">
+        <v>62</v>
+      </c>
+      <c r="B69" t="s">
         <v>31</v>
       </c>
-      <c r="B40" t="s">
-        <v>37</v>
-      </c>
-      <c r="C40">
+      <c r="C69">
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41">
-        <v>32</v>
-      </c>
-      <c r="B41" t="s">
-        <v>38</v>
-      </c>
-      <c r="C41">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A70">
+        <v>63</v>
+      </c>
+      <c r="B70" t="s">
+        <v>73</v>
+      </c>
+      <c r="C70">
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42">
-        <v>33</v>
-      </c>
-      <c r="B42" t="s">
-        <v>39</v>
-      </c>
-      <c r="C42">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A71">
+        <v>64</v>
+      </c>
+      <c r="B71" t="s">
+        <v>74</v>
+      </c>
+      <c r="C71">
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43">
-        <v>34</v>
-      </c>
-      <c r="B43" t="s">
-        <v>40</v>
-      </c>
-      <c r="C43">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A72">
+        <v>65</v>
+      </c>
+      <c r="B72" t="s">
+        <v>75</v>
+      </c>
+      <c r="C72">
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44">
-        <v>35</v>
-      </c>
-      <c r="B44" t="s">
-        <v>41</v>
-      </c>
-      <c r="C44">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A73">
+        <v>66</v>
+      </c>
+      <c r="B73" t="s">
+        <v>76</v>
+      </c>
+      <c r="C73">
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45">
-        <v>36</v>
-      </c>
-      <c r="B45" t="s">
-        <v>42</v>
-      </c>
-      <c r="C45">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A74">
+        <v>67</v>
+      </c>
+      <c r="B74" t="s">
+        <v>77</v>
+      </c>
+      <c r="C74">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A75">
+        <v>68</v>
+      </c>
+      <c r="B75" t="s">
+        <v>71</v>
+      </c>
+      <c r="C75">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A76">
+        <v>69</v>
+      </c>
+      <c r="B76" t="s">
+        <v>78</v>
+      </c>
+      <c r="C76">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A77">
+        <v>70</v>
+      </c>
+      <c r="B77" t="s">
+        <v>79</v>
+      </c>
+      <c r="C77">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A78">
+        <v>71</v>
+      </c>
+      <c r="B78" t="s">
+        <v>70</v>
+      </c>
+      <c r="C78">
         <v>6</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46">
-        <v>37</v>
-      </c>
-      <c r="B46" t="s">
-        <v>43</v>
-      </c>
-      <c r="C46">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A79">
+        <v>72</v>
+      </c>
+      <c r="B79" t="s">
+        <v>68</v>
+      </c>
+      <c r="C79">
         <v>6</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47">
-        <v>38</v>
-      </c>
-      <c r="B47" t="s">
-        <v>14</v>
-      </c>
-      <c r="C47">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A80">
+        <v>73</v>
+      </c>
+      <c r="B80" t="s">
+        <v>72</v>
+      </c>
+      <c r="C80">
         <v>6</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48">
-        <v>39</v>
-      </c>
-      <c r="B48" t="s">
-        <v>44</v>
-      </c>
-      <c r="C48">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49">
-        <v>40</v>
-      </c>
-      <c r="B49" t="s">
-        <v>45</v>
-      </c>
-      <c r="C49">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50">
-        <v>41</v>
-      </c>
-      <c r="B50" t="s">
-        <v>46</v>
-      </c>
-      <c r="C50">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51">
-        <v>42</v>
-      </c>
-      <c r="B51" t="s">
-        <v>47</v>
-      </c>
-      <c r="C51">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52">
-        <v>43</v>
-      </c>
-      <c r="B52" t="s">
-        <v>48</v>
-      </c>
-      <c r="C52">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53">
-        <v>44</v>
-      </c>
-      <c r="B53" t="s">
-        <v>49</v>
-      </c>
-      <c r="C53">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54">
-        <v>45</v>
-      </c>
-      <c r="B54" t="s">
-        <v>50</v>
-      </c>
-      <c r="C54">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55">
-        <v>46</v>
-      </c>
-      <c r="B55" t="s">
-        <v>51</v>
-      </c>
-      <c r="C55">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56">
-        <v>47</v>
-      </c>
-      <c r="B56" t="s">
-        <v>52</v>
-      </c>
-      <c r="C56">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57">
-        <v>48</v>
-      </c>
-      <c r="B57" t="s">
-        <v>14</v>
-      </c>
-      <c r="C57">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58">
-        <v>49</v>
-      </c>
-      <c r="B58" t="s">
-        <v>53</v>
-      </c>
-      <c r="C58">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59">
-        <v>50</v>
-      </c>
-      <c r="B59" t="s">
-        <v>54</v>
-      </c>
-      <c r="C59">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60">
-        <v>51</v>
-      </c>
-      <c r="B60" t="s">
-        <v>55</v>
-      </c>
-      <c r="C60">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61">
-        <v>52</v>
-      </c>
-      <c r="B61" t="s">
-        <v>56</v>
-      </c>
-      <c r="C61">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62">
-        <v>53</v>
-      </c>
-      <c r="B62" t="s">
-        <v>57</v>
-      </c>
-      <c r="C62">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63">
-        <v>54</v>
-      </c>
-      <c r="B63" t="s">
-        <v>58</v>
-      </c>
-      <c r="C63">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A64">
-        <v>55</v>
-      </c>
-      <c r="B64" t="s">
-        <v>59</v>
-      </c>
-      <c r="C64">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65">
-        <v>56</v>
-      </c>
-      <c r="B65" t="s">
-        <v>60</v>
-      </c>
-      <c r="C65">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A66">
-        <v>57</v>
-      </c>
-      <c r="B66" t="s">
-        <v>61</v>
-      </c>
-      <c r="C66">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A67">
-        <v>58</v>
-      </c>
-      <c r="B67" t="s">
-        <v>62</v>
-      </c>
-      <c r="C67">
-        <v>8</v>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A81">
+        <v>74</v>
+      </c>
+      <c r="B81" t="s">
+        <v>67</v>
+      </c>
+      <c r="C81">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A82">
+        <v>75</v>
+      </c>
+      <c r="B82" t="s">
+        <v>31</v>
+      </c>
+      <c r="C82">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A83">
+        <v>76</v>
+      </c>
+      <c r="B83" t="s">
+        <v>73</v>
+      </c>
+      <c r="C83">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A84">
+        <v>77</v>
+      </c>
+      <c r="B84" t="s">
+        <v>74</v>
+      </c>
+      <c r="C84">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A85">
+        <v>78</v>
+      </c>
+      <c r="B85" t="s">
+        <v>75</v>
+      </c>
+      <c r="C85">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A86">
+        <v>79</v>
+      </c>
+      <c r="B86" t="s">
+        <v>76</v>
+      </c>
+      <c r="C86">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A87">
+        <v>80</v>
+      </c>
+      <c r="B87" t="s">
+        <v>77</v>
+      </c>
+      <c r="C87">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A88">
+        <v>81</v>
+      </c>
+      <c r="B88" t="s">
+        <v>71</v>
+      </c>
+      <c r="C88">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A89">
+        <v>82</v>
+      </c>
+      <c r="B89" t="s">
+        <v>78</v>
+      </c>
+      <c r="C89">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A90">
+        <v>83</v>
+      </c>
+      <c r="B90" t="s">
+        <v>79</v>
+      </c>
+      <c r="C90">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1792,658 +2085,658 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C59"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="B1" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="C1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C10">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C11">
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="C12">
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="C13">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C14">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C15">
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="C16">
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C17">
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="C18">
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="C19">
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="C20">
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C21">
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="C22">
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="C23">
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="C24">
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="C25">
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="C26">
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="C27">
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="C28">
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="C29">
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="C30">
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="C31">
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C32">
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="C33">
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="C34">
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="C35">
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="C36">
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="C37">
         <v>6</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="C38">
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C39">
         <v>6</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="C40">
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="C41">
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C42">
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="C43">
         <v>7</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C44">
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="C45">
         <v>7</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="C46">
         <v>7</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="C47">
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="C48">
         <v>7</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C49">
         <v>7</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="C50">
         <v>7</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="C51">
         <v>7</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="C52">
         <v>7</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="C53">
         <v>7</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="C54">
         <v>7</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C55">
         <v>8</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="C56">
         <v>8</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="C57">
         <v>8</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="C58">
         <v>8</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="C59">
         <v>8</v>

</xml_diff>